<commit_message>
Base the Lab 04 SMath plot on the Excel chart
The worksheet picture is now a render of the Excel workbook's chart
instead of a separate matplotlib plot, and the chart's markers, colors,
and axis ranges are set explicitly so both look the same.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VscspVnmobd9ZrHwQsr1zU
</commit_message>
<xml_diff>
--- a/labs/lab04_flowrate/Lab_04_-_Flowrate_Plot.xlsx
+++ b/labs/lab04_flowrate/Lab_04_-_Flowrate_Plot.xlsx
@@ -126,7 +126,7 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="13"/>
+  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -145,6 +145,7 @@
     </title>
     <plotArea>
       <scatterChart>
+        <scatterStyle val="lineMarker"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
@@ -159,8 +160,15 @@
           </spPr>
           <marker>
             <symbol val="circle"/>
+            <size val="7"/>
             <spPr>
+              <a:solidFill>
+                <a:srgbClr val="1F77B4"/>
+              </a:solidFill>
               <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="1F77B4"/>
+                </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -180,6 +188,14 @@
                 <f>'Flowrates (GPM)'!$D$2:$D$7</f>
               </numRef>
             </plus>
+            <spPr>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="1F77B4"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
           </errBars>
           <xVal>
             <numRef>
@@ -205,9 +221,16 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="circle"/>
+            <symbol val="square"/>
+            <size val="7"/>
             <spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF7F0E"/>
+              </a:solidFill>
               <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="FF7F0E"/>
+                </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -227,6 +250,14 @@
                 <f>'Flowrates (GPM)'!$F$2:$F$7</f>
               </numRef>
             </plus>
+            <spPr>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FF7F0E"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
           </errBars>
           <xVal>
             <numRef>
@@ -252,9 +283,16 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="circle"/>
+            <symbol val="triangle"/>
+            <size val="7"/>
             <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2CA02C"/>
+              </a:solidFill>
               <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="2CA02C"/>
+                </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -274,6 +312,14 @@
                 <f>'Flowrates (GPM)'!$H$2:$H$7</f>
               </numRef>
             </plus>
+            <spPr>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="2CA02C"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
           </errBars>
           <xVal>
             <numRef>
@@ -299,9 +345,16 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="circle"/>
+            <symbol val="diamond"/>
+            <size val="7"/>
             <spPr>
+              <a:solidFill>
+                <a:srgbClr val="D62728"/>
+              </a:solidFill>
               <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="D62728"/>
+                </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -321,6 +374,14 @@
                 <f>'Flowrates (GPM)'!$J$2:$J$7</f>
               </numRef>
             </plus>
+            <spPr>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="D62728"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
           </errBars>
           <xVal>
             <numRef>
@@ -346,9 +407,16 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="circle"/>
+            <symbol val="x"/>
+            <size val="7"/>
             <spPr>
+              <a:solidFill>
+                <a:srgbClr val="9467BD"/>
+              </a:solidFill>
               <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="9467BD"/>
+                </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -368,6 +436,14 @@
                 <f>'Flowrates (GPM)'!$L$2:$L$7</f>
               </numRef>
             </plus>
+            <spPr>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="9467BD"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
           </errBars>
           <xVal>
             <numRef>
@@ -393,9 +469,16 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="circle"/>
+            <symbol val="star"/>
+            <size val="7"/>
             <spPr>
+              <a:solidFill>
+                <a:srgbClr val="8C564B"/>
+              </a:solidFill>
               <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="8C564B"/>
+                </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -415,6 +498,14 @@
                 <f>'Flowrates (GPM)'!$N$2:$N$7</f>
               </numRef>
             </plus>
+            <spPr>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="8C564B"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
           </errBars>
           <xVal>
             <numRef>
@@ -434,6 +525,8 @@
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="8"/>
+          <min val="2"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -453,14 +546,18 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="20"/>
+        <majorUnit val="1"/>
       </valAx>
       <valAx>
         <axId val="20"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="11"/>
+          <min val="0"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -474,15 +571,17 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Measured Flowrate (GPM)</a:t>
+                  <a:t>Measured Flowrate, Q (GPM)</a:t>
                 </a:r>
               </a:p>
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <majorUnit val="1"/>
       </valAx>
     </plotArea>
     <legend>
@@ -503,7 +602,7 @@
       <row>9</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6480000" cy="3960000"/>
+    <ext cx="7200000" cy="4320000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>

</xml_diff>